<commit_message>
Implement lenient TCP flag comparison - flag order doesn't matter
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/cuongnhhe186494/OverallSummary.xlsx
+++ b/Submit/Results/cuongnhhe186494/OverallSummary.xlsx
@@ -41,9 +41,6 @@
   </x:si>
   <x:si>
     <x:t>TC2_Send</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
   </x:si>
   <x:si>
     <x:t>TC3_ReqResNotC</x:t>
@@ -473,12 +470,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>6</x:v>
@@ -490,12 +487,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
       <x:c r="A5" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>6</x:v>
@@ -507,7 +504,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Fix golden DLL file override - remove old appsettings + clean directories before copying
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/cuongnhhe186494/OverallSummary.xlsx
+++ b/Submit/Results/cuongnhhe186494/OverallSummary.xlsx
@@ -41,12 +41,6 @@
   </x:si>
   <x:si>
     <x:t>TC2_Send</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PASS</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
   </x:si>
   <x:si>
     <x:t>TC3_ReqResNotC</x:t>
@@ -467,21 +461,21 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C3" s="0">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D3" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>6</x:v>
@@ -493,12 +487,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
       <x:c r="A5" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>6</x:v>
@@ -510,7 +504,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>